<commit_message>
31Aug Deployment - For Avi Machine
</commit_message>
<xml_diff>
--- a/nseIndia/exportedData/CorporateActions.xlsx
+++ b/nseIndia/exportedData/CorporateActions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,7 +503,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MUNJALAU</t>
+          <t>TRIVENI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -518,22 +518,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dividend - Re 1 Per Sh</t>
+          <t>Dividend - Rs 2.50 Per Share</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Munjal Auto Industries Limited</t>
+          <t>Triveni Engineering &amp; Industries Limited</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>INE672B01024</t>
+          <t>INE256C01024</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -571,7 +571,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MURUDCERA</t>
+          <t>ALIVUS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -586,22 +586,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Dividend - Rs 0.50 Per Share</t>
+          <t>Dividend - Rs 5 Per Share</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -621,12 +621,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Murudeshwar Ceramics Limited</t>
+          <t>Alivus Life Sciences Limited</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>INE692B01014</t>
+          <t>INE03Q201024</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GPIL</t>
+          <t>PAVNAIND</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -654,22 +654,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Dividend - Re 1 Per Share</t>
+          <t>Face Value Split (Sub-Division) - From Rs 10/- Per Share To Re 1/- Per Share</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>16-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Godawari Power And Ispat limited</t>
+          <t>Pavna Industries Limited</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>INE177H01013</t>
+          <t>INE07S101020</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>KANPRPLA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -722,22 +722,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dividend - Rs 0.90 Per Share</t>
+          <t>Dividend - Re 0.90 Per Share</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Bharat Electronics Limited</t>
+          <t>Kanpur Plastipack Limited</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>INE263A01016</t>
+          <t>INE694E01014</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>MMP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -790,22 +790,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dividend - Rs 0.90 Per Share</t>
+          <t>Dividend - Rs 2 Per Share</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -825,12 +825,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Minda Corporation Limited</t>
+          <t>MMP Industries Limited</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>INE842C01013</t>
+          <t>INE511Y01018</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -843,7 +843,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TFCILTD</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -863,17 +863,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Dividend - Rs 3 Per Share</t>
+          <t>Dividend - Re 0.30 Per Share</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Tourism Finance Corporation of India Limited</t>
+          <t>Patel Integrated Logistics Limited</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>INE305A01015</t>
+          <t>INE529D01014</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -911,7 +911,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NMDC</t>
+          <t>TRITURBINE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -931,17 +931,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dividend - Re 1 Per Share</t>
+          <t>Dividend - Rs 2 Per Share</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>01-Sep-2025</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -961,12 +961,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>NMDC Limited</t>
+          <t>Triveni Turbine Limited</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>INE584A01023</t>
+          <t>INE152M01016</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ELECTCAST</t>
+          <t>PANAMAPET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -994,22 +994,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Dividend - Rs 1.40 Per Share</t>
+          <t>Dividend - Rs 3 Per Share</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>15-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1029,12 +1029,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Electrosteel Castings Limited</t>
+          <t>Panama Petrochem Limited</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>INE086A01029</t>
+          <t>INE305C01011</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,7 +1047,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>YASHO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1067,17 +1067,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Dividend - Rs 5.5 Per Share</t>
+          <t>Dividend - Re 0.50 Per Share</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1097,12 +1097,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Reliance Industries Limited</t>
+          <t>Yasho Industries Limited</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>INE002A01018</t>
+          <t>INE616Z01012</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1115,7 +1115,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KRYSTAL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1140,12 +1140,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>15-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1165,12 +1165,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Mangalam Cement Limited</t>
+          <t>Krystal Integrated Services Limited</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>INE347A01017</t>
+          <t>INE0QN801017</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>JINDRILL</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1198,22 +1198,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Dividend - Re 1 Per Share</t>
+          <t>Dividend - Rs 2 Per Share</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1233,12 +1233,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Jindal Drilling And Industries Limited</t>
+          <t>MODISON LIMITED</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>INE742C01031</t>
+          <t>INE737D01021</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1251,7 +1251,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALKALI</t>
+          <t>TPLPLASTEH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1266,22 +1266,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Dividend - Re 0.50 Per Share</t>
+          <t>Dividend - Re 1 Per Share</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1301,12 +1301,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Alkali Metals Limited</t>
+          <t>TPL Plastech Limited</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>INE773I01017</t>
+          <t>INE413G01014</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1319,7 +1319,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LGBBROSLTD</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1334,22 +1334,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Dividend - Rs 20 Per Share</t>
+          <t>Dividend - Rs 0.80 Per Share</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>LG Balakrishnan &amp; Bros Limited</t>
+          <t>Hikal Limited</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>INE337A01034</t>
+          <t>INE475B01014</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1387,7 +1387,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1407,17 +1407,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Dividend - Rs 2.60 Per Share</t>
+          <t>Dividend - Rs 2.25 Per Share</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>REC Limited</t>
+          <t>Tribhovandas Bhimji Zaveri Limited</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>INE020B01018</t>
+          <t>INE760L01018</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1455,7 +1455,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MAHSEAMLES</t>
+          <t>GNFC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1470,22 +1470,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Dividend - Rs 10 Per Sh</t>
+          <t>Dividend - Rs 18 Per Share</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1505,12 +1505,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Maharashtra Seamless Limited</t>
+          <t>Gujarat Narmada Valley Fertilizers and Chemicals Limited</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>INE271B01025</t>
+          <t>INE113A01013</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1523,7 +1523,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>AJMERA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1543,17 +1543,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Dividend - Rs 10 Per Share</t>
+          <t>Dividend - Rs 4.50 Per Share</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Venky's (India) Limited</t>
+          <t>Ajmera Realty &amp; Infra India Limited</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>INE398A01010</t>
+          <t>INE298G01027</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1591,7 +1591,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ACE</t>
+          <t>RATNAMANI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1611,17 +1611,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Dividend - Rs 2 Per Share</t>
+          <t>Dividend - Rs 14 Per Share</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>02-Sep-2025</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1641,12 +1641,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Action Construction Equipment Limited</t>
+          <t>Ratnamani Metals &amp; Tubes Limited</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>INE731H01025</t>
+          <t>INE703B01027</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1659,7 +1659,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MANGCHEFER</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1674,22 +1674,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Dividend - Rs 1.50 Per Share</t>
+          <t>Dividend - Rs 1.25 Per Share</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>04-Sep-2025</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>14-Aug-2025</t>
+          <t>04-Sep-2025</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1709,12 +1709,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Mangalore Chemicals &amp; Fertilizers Limited</t>
+          <t>Oil &amp; Natural Gas Corporation Limited</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>INE558B01017</t>
+          <t>INE213A01011</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1723,142 +1723,6 @@
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WSTCSTPAPR</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>EQ</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Dividend - Rs 5 Per Share</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>14-Aug-2025</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>14-Aug-2025</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>West Coast Paper Mills Limited</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>INE976A01021</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>EXCELINDUS</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>EQ</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Dividend - Rs 13.75 Per Share</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>14-Aug-2025</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>14-Aug-2025</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Excel Industries Limited</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>INE369A01029</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>